<commit_message>
feat(compart): ajout d'un bouton pour changer ajuster l'echelle
[40][DONE]
vu les écart que j'ai entre mes devise j'ai décider d'ajouter un bouton
pour comparé. le consepete mettre tous en Base 100 pour une meuilleur
comparaison. Un hover sur les points indique la valeur de base
</commit_message>
<xml_diff>
--- a/doc/journal_de_travail.xlsx
+++ b/doc/journal_de_travail.xlsx
@@ -10,8 +10,8 @@
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$6</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +43,20 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +117,60 @@
         <bgColor rgb="FFE65100"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+        <bgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF5FC"/>
+        <bgColor rgb="00EEF5FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00455A64"/>
+        <bgColor rgb="00455A64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006A1B9A"/>
+        <bgColor rgb="006A1B9A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E8FA"/>
+        <bgColor rgb="00D6E8FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001565C0"/>
+        <bgColor rgb="001565C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E7D32"/>
+        <bgColor rgb="002E7D32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E65100"/>
+        <bgColor rgb="00E65100"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -118,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -146,6 +212,31 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -401,6 +492,1161 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart18.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart19.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
@@ -580,6 +1826,349 @@
     <legend>
       <legendPos val="r"/>
       <overlay val="0"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart20.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart21.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart22.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -946,6 +2535,580 @@
     <legend>
       <legendPos val="r"/>
       <overlay val="0"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1038,6 +3201,402 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="7" name="Chart 7"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="8" name="Chart 8"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId8"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="9" name="Chart 9"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId9"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="10" name="Chart 10"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId10"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="11" name="Chart 11"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId11"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="12" name="Chart 12"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId12"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="13" name="Chart 13"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId13"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="14" name="Chart 14"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId14"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="15" name="Chart 15"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId15"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="16" name="Chart 16"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId16"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="17" name="Chart 17"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId17"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="18" name="Chart 18"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId18"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="19" name="Chart 19"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId19"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="20" name="Chart 20"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId20"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="21" name="Chart 21"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId21"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="22" name="Chart 22"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId22"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1335,12 +3894,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="1"/>
     <col width="18" customWidth="1" style="12" min="2" max="2"/>
-    <col width="217.85546875" bestFit="1" customWidth="1" style="12" min="3" max="3"/>
+    <col width="75" bestFit="1" customWidth="1" style="12" min="3" max="3"/>
     <col width="16" customWidth="1" style="12" min="4" max="4"/>
     <col width="12" customWidth="1" style="12" min="5" max="5"/>
   </cols>
@@ -1373,469 +3932,721 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>24/08/2026</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr"/>
+      <c r="B3" s="15" t="inlineStr"/>
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>commit initial</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>[2]</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr"/>
+      <c r="B4" s="15" t="inlineStr"/>
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>explication du projet (CdC, Carnet de voyage, projet hanbook)</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>[105]</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr"/>
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Tâche</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>écriture du lisez-moi + structure de fichiers</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>[21]</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr"/>
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>Tâche</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>ajoute le script d'export pdf aux fichiers ignorés</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>[19]</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr"/>
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>Tâche</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>début du rapport</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>[30]</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr"/>
+      <c r="B8" s="17" t="inlineStr"/>
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>2h57 (177 min)</t>
         </is>
       </c>
-      <c r="E8" s="5" t="n"/>
+      <c r="E8" s="17" t="inlineStr"/>
     </row>
-    <row r="9"/>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+    </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>31/08/2026</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr"/>
+      <c r="B11" s="15" t="inlineStr"/>
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>absence</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>[180]</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr"/>
+      <c r="B12" s="17" t="inlineStr"/>
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>3h00 (180 min)</t>
         </is>
       </c>
-      <c r="E12" s="5" t="n"/>
+      <c r="E12" s="17" t="inlineStr"/>
     </row>
-    <row r="13"/>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+    </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>01/09/2026</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr"/>
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>Étoffe les objectifs produit et pédagogiques, décrit le domaine (cryptomonnaies, 5 séries cohérentes, interface Binance) et remplace la planification par une version complète (méthodologie, sprints, répartition des tâches, risques).</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>[30]</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr"/>
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>Ajoute l'analyse fonctionnelle basée sur les user stories du projet Kanban GitHub, avec besoins fonctionnels et non-fonctionnels, ainsi que les contraintes techniques.</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>[30]</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr"/>
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>Supprime la section répartition des tâches et toutes les mentions d'équipe ou de binôme dans le rapport. Adapte les formulations au singulier et renumérote les sous-sections de la planification.</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>[15]</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr"/>
+      <c r="B18" s="17" t="inlineStr"/>
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>1h15 (75 min)</t>
         </is>
       </c>
-      <c r="E18" s="5" t="n"/>
+      <c r="E18" s="17" t="inlineStr"/>
     </row>
-    <row r="19"/>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+    </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>07/09/2026</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="A21" s="14" t="inlineStr"/>
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>ajoute la fenêtre principale avec le panneau graphique et les checkboxes des séries</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>[12]</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr"/>
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>Refactorisation</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>génère les checkboxes des séries avec LINQ</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>[18]</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr"/>
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>ajoute le record immuable CryptoSeries</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>[26]</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="A24" s="14" t="inlineStr"/>
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>ajoute le catalogue des 5 séries crypto</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>[12]</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr"/>
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t>Refactorisation</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>génère les checkboxes avec LINQ via des méthodes d'extension</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>[42]</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>[40]</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr"/>
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>Fonctionnalité</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>ajoute ScottPlot pour afficher un graphique X/Y à gauche</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>[25min]</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>[25]</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>WIP feat(data): ajoute l'importeur de séries depuis un fichier CSV</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>[20]</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr"/>
+      <c r="B27" s="20" t="inlineStr">
+        <is>
+          <t>Fonctionnalité</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>ajoute l'importeur de séries depuis un fichier CSV</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>[15]</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>WIP feat(gui): branche l'import CSV dans la fenêtre principale</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
+      <c r="A28" s="14" t="inlineStr"/>
+      <c r="B28" s="20" t="inlineStr">
+        <is>
+          <t>Fonctionnalité</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>branche l'import CSV dans la fenêtre principale</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>[18]</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="14" t="inlineStr">
         <is>
           <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n"/>
-      <c r="B29" s="5" t="n"/>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr"/>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>Tâche</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>enregistre l'import CSV dans le journal</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr"/>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>Tâche</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>ajoute le script get_commit</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr"/>
+      <c r="B31" s="20" t="inlineStr">
+        <is>
+          <t>Fonctionnalité</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>ajoute l'importeur de séries depuis un fichier CSV</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>[WIP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr"/>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>Fonctionnalité</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>branche l'import CSV dans la fenêtre principale</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>[WIP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr"/>
+      <c r="B33" s="17" t="inlineStr"/>
+      <c r="C33" s="18" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>2h53 (173 min)</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="n"/>
+      <c r="D33" s="18" t="inlineStr">
+        <is>
+          <t>2h56 (176 min)</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr"/>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>Tâche</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>data de base pour le bon fonctionnement de l'app</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>[15]</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr"/>
+      <c r="B37" s="20" t="inlineStr">
+        <is>
+          <t>Fonctionnalité</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>importe les data depuis une sources Correction possibilité de réécrire sur les date</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>[25]</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr"/>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>Tâche</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>ajout de data pour mes tests d'importation</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>[10]</t>
+        </is>
+      </c>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr"/>
+      <c r="B39" s="20" t="inlineStr">
+        <is>
+          <t>Fonctionnalité</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>sauvegarde dans SQLite les datas. Importation: ajout les data ne fait pas de chevauchement</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>[20]</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr"/>
+      <c r="B40" s="17" t="inlineStr"/>
+      <c r="C40" s="18" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="D40" s="18" t="inlineStr">
+        <is>
+          <t>1h10 (70 min)</t>
+        </is>
+      </c>
+      <c r="E40" s="17" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E28"/>
-  <mergeCells count="4">
+  <autoFilter ref="A1:E41"/>
+  <mergeCells count="6">
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A37:E37"/>
     <mergeCell ref="A14:E14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1848,7 +4659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="12" min="1" max="1"/>
@@ -1858,42 +4669,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="22" t="inlineStr">
         <is>
           <t>Total (min)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="22" t="inlineStr">
         <is>
           <t>Total (h)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="22" t="inlineStr">
         <is>
           <t>Total (h:min)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="22" t="inlineStr">
         <is>
           <t>Indicateur</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="22" t="inlineStr">
         <is>
           <t>Valeur</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="23" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="23" t="inlineStr">
         <is>
           <t>Cumul (h)</t>
         </is>
@@ -1916,13 +4727,13 @@
           <t>2h57</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>Jours suivis</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1950,14 +4761,14 @@
           <t>3h00</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="23" t="inlineStr">
         <is>
           <t>Temps total</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>9h27</t>
+          <t>11h18</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1986,14 +4797,14 @@
           <t>1h15</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="F4" s="23" t="inlineStr">
         <is>
           <t>Moyenne / jour</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2h22</t>
+          <t>2h16</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -2012,17 +4823,17 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C5" t="n">
-        <v>2.88</v>
+        <v>2.93</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2h53</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
+          <t>2h56</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
         <is>
           <t>Jour le plus chargé</t>
         </is>
@@ -2038,11 +4849,37 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>10.08</v>
+        <v>10.13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>70</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1h10</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>11.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D5"/>
+  <autoFilter ref="A1:D6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor(ALL): sortire du mainPage.cs le code
[22][WIP]
</commit_message>
<xml_diff>
--- a/doc/journal_de_travail.xlsx
+++ b/doc/journal_de_travail.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$6</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1954,7 +1954,6 @@
 
 <file path=xl/charts/chart21.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -2066,6 +2065,469 @@
 </file>
 
 <file path=xl/charts/chart22.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart23.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart24.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart25.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart26.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -3602,6 +4064,94 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="23" name="Chart 23"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId23"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="24" name="Chart 24"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId24"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="25" name="Chart 25"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId25"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="26" name="Chart 26"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId26"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -3894,7 +4444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="1"/>
@@ -4618,29 +5168,98 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="inlineStr"/>
-      <c r="B40" s="17" t="inlineStr"/>
-      <c r="C40" s="18" t="inlineStr">
-        <is>
-          <t>Total du jour</t>
-        </is>
-      </c>
-      <c r="D40" s="18" t="inlineStr">
-        <is>
-          <t>1h10 (70 min)</t>
-        </is>
-      </c>
-      <c r="E40" s="17" t="inlineStr"/>
+      <c r="A40" s="14" t="inlineStr"/>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>Fonctionnalité</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>vu les écart que j'ai entre mes devise j'ai décider d'ajouter un bouton pour comparé. le consepete mettre tous en Base 100 pour une meuilleur comparaison. Un hover sur les points indique la valeur de base</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>[40]</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
+      <c r="A41" s="14" t="inlineStr"/>
+      <c r="B41" s="20" t="inlineStr">
+        <is>
+          <t>Fonctionnalité</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Structure basique tests basique pas forcement fonctionnel</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>[20]</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>[WIP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr"/>
+      <c r="B42" s="19" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>discution</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>[25]</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr"/>
+      <c r="B43" s="17" t="inlineStr"/>
+      <c r="C43" s="18" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="D43" s="18" t="inlineStr">
+        <is>
+          <t>2h35 (155 min)</t>
+        </is>
+      </c>
+      <c r="E43" s="17" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E41"/>
+  <autoFilter ref="A1:E44"/>
   <mergeCells count="6">
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A20:E20"/>
@@ -4768,7 +5387,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>11h18</t>
+          <t>12h43</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -4804,7 +5423,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2h16</t>
+          <t>2h33</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -4859,14 +5478,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>70</v>
+        <v>155</v>
       </c>
       <c r="C6" t="n">
-        <v>1.17</v>
+        <v>2.58</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1h10</t>
+          <t>2h35</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -4875,7 +5494,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>11.3</v>
+        <v>12.72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Chor(JNR): mise a jour
[2][DONE]
</commit_message>
<xml_diff>
--- a/doc/journal_de_travail.xlsx
+++ b/doc/journal_de_travail.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$6</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -2416,7 +2416,6 @@
 
 <file path=xl/charts/chart25.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -2528,6 +2527,238 @@
 </file>
 
 <file path=xl/charts/chart26.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart27.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart28.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -4152,6 +4383,50 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="27" name="Chart 27"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId27"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="28" name="Chart 28"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId28"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -4444,7 +4719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="1"/>
@@ -5237,29 +5512,52 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="inlineStr"/>
-      <c r="B43" s="17" t="inlineStr"/>
-      <c r="C43" s="18" t="inlineStr">
-        <is>
-          <t>Total du jour</t>
-        </is>
-      </c>
-      <c r="D43" s="18" t="inlineStr">
-        <is>
-          <t>2h35 (155 min)</t>
-        </is>
-      </c>
-      <c r="E43" s="17" t="inlineStr"/>
+      <c r="A43" s="14" t="inlineStr"/>
+      <c r="B43" s="21" t="inlineStr">
+        <is>
+          <t>Refactorisation</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>sortire du mainPage.cs le code</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>[22]</t>
+        </is>
+      </c>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>[WIP]</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
+      <c r="A44" s="17" t="inlineStr"/>
+      <c r="B44" s="17" t="inlineStr"/>
+      <c r="C44" s="18" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="D44" s="18" t="inlineStr">
+        <is>
+          <t>2h57 (177 min)</t>
+        </is>
+      </c>
+      <c r="E44" s="17" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E44"/>
+  <autoFilter ref="A1:E45"/>
   <mergeCells count="6">
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A20:E20"/>
@@ -5387,7 +5685,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>12h43</t>
+          <t>13h05</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -5423,7 +5721,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2h33</t>
+          <t>2h37</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -5478,14 +5776,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>155</v>
+        <v>177</v>
       </c>
       <c r="C6" t="n">
-        <v>2.58</v>
+        <v>2.95</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2h35</t>
+          <t>2h57</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -5494,7 +5792,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>12.72</v>
+        <v>13.08</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
perf(plot): SignalXY, survol fenêtré et couleurs fixes par série
Le rendu devenait poussif avec les 39 000 bougies par série : Scatter
redessinait un marqueur par point à chaque zoom. Passage à SignalXY, qui
ne trace que la partie visible, et recherche du point survolé limitée à
une fenêtre trouvée par dichotomie au lieu de reprojeter toute la série.
Les couleurs viennent maintenant d'une palette indexée sur la position de
la série, pour que masquer une courbe ne recolore plus les autres.
</commit_message>
<xml_diff>
--- a/doc/journal_de_travail.xlsx
+++ b/doc/journal_de_travail.xlsx
@@ -10,8 +10,8 @@
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$7</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -2647,7 +2647,6 @@
 
 <file path=xl/charts/chart27.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -2792,6 +2791,14 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
           <cat>
             <numRef>
               <f>'Tableau de bord'!$A$2:$A$6</f>
@@ -2807,6 +2814,119 @@
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart29.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -3041,6 +3161,117 @@
     <legend>
       <legendPos val="r"/>
       <overlay val="0"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart30.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -4427,6 +4658,50 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="29" name="Chart 29"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId29"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="30" name="Chart 30"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId30"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -4719,7 +4994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="1"/>
@@ -5535,34 +5810,175 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="inlineStr"/>
-      <c r="B44" s="17" t="inlineStr"/>
-      <c r="C44" s="18" t="inlineStr">
-        <is>
-          <t>Total du jour</t>
-        </is>
-      </c>
-      <c r="D44" s="18" t="inlineStr">
-        <is>
-          <t>2h57 (177 min)</t>
-        </is>
-      </c>
-      <c r="E44" s="17" t="inlineStr"/>
+      <c r="A44" s="14" t="inlineStr"/>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>Tâche</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>mise a jour</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
+      <c r="A45" s="17" t="inlineStr"/>
+      <c r="B45" s="17" t="inlineStr"/>
+      <c r="C45" s="18" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="D45" s="18" t="inlineStr">
+        <is>
+          <t>2h59 (179 min)</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="14" t="inlineStr"/>
+      <c r="B48" s="20" t="inlineStr">
+        <is>
+          <t>Fonctionnalité</t>
+        </is>
+      </c>
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>script qui récupère directement sur l'interface</t>
+        </is>
+      </c>
+      <c r="D48" s="14" t="inlineStr">
+        <is>
+          <t>[35]</t>
+        </is>
+      </c>
+      <c r="E48" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr"/>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>Tâche</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>Pourquoi j'ai fait ça: les Json peuvent être généré avec le script du commit d'avant l'il n'y a donc plus d'utilité.</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="inlineStr">
+        <is>
+          <t>[10]</t>
+        </is>
+      </c>
+      <c r="E49" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr"/>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>Tâche</t>
+        </is>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>modification du gitignore</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="inlineStr">
+        <is>
+          <t>[?]</t>
+        </is>
+      </c>
+      <c r="E50" s="14" t="inlineStr">
+        <is>
+          <t>[?]</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr"/>
+      <c r="B51" s="15" t="inlineStr"/>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>mise à jour(base de données): up to 190000 data</t>
+        </is>
+      </c>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>[5]</t>
+        </is>
+      </c>
+      <c r="E51" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr"/>
+      <c r="B52" s="17" t="inlineStr"/>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>0h50 (50 min)</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E45"/>
-  <mergeCells count="6">
+  <autoFilter ref="A1:E53"/>
+  <mergeCells count="7">
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A47:E47"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A14:E14"/>
   </mergeCells>
@@ -5576,7 +5992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="12" min="1" max="1"/>
@@ -5650,7 +6066,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -5685,7 +6101,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>13h05</t>
+          <t>13h57</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -5721,7 +6137,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2h37</t>
+          <t>2h20</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -5776,14 +6192,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C6" t="n">
-        <v>2.95</v>
+        <v>2.98</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2h57</t>
+          <t>2h59</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -5792,11 +6208,37 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>13.08</v>
+        <v>13.12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0h50</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>13.95</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D6"/>
+  <autoFilter ref="A1:D7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
doc(MAJ): mise a jour du rapport et du JNR
[10][DONE]
</commit_message>
<xml_diff>
--- a/doc/journal_de_travail.xlsx
+++ b/doc/journal_de_travail.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$7</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -56,7 +56,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -171,6 +171,12 @@
         <bgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00558B2F"/>
+        <bgColor rgb="00558B2F"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -184,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -237,6 +243,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2878,7 +2887,6 @@
 
 <file path=xl/charts/chart29.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -3202,6 +3210,14 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
           <cat>
             <numRef>
               <f>'Tableau de bord'!$A$2:$A$7</f>
@@ -3217,6 +3233,1043 @@
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart31.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart32.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart33.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart34.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart35.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart36.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart37.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart38.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart39.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -3459,6 +4512,117 @@
     <legend>
       <legendPos val="r"/>
       <overlay val="0"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart40.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -4702,6 +5866,226 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="31" name="Chart 31"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId31"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="32" name="Chart 32"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId32"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="33" name="Chart 33"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId33"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="34" name="Chart 34"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId34"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="35" name="Chart 35"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId35"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="36" name="Chart 36"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId36"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="37" name="Chart 37"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId37"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="38" name="Chart 38"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId38"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="39" name="Chart 39"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId39"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="40" name="Chart 40"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId40"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -4994,7 +6378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="1"/>
@@ -5921,12 +7305,12 @@
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>[?]</t>
+          <t>[1]</t>
         </is>
       </c>
       <c r="E50" s="14" t="inlineStr">
         <is>
-          <t>[?]</t>
+          <t>[DONE]</t>
         </is>
       </c>
     </row>
@@ -5950,29 +7334,94 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="17" t="inlineStr"/>
-      <c r="B52" s="17" t="inlineStr"/>
-      <c r="C52" s="18" t="inlineStr">
-        <is>
-          <t>Total du jour</t>
-        </is>
-      </c>
-      <c r="D52" s="18" t="inlineStr">
-        <is>
-          <t>0h50 (50 min)</t>
-        </is>
-      </c>
-      <c r="E52" s="17" t="inlineStr"/>
+      <c r="A52" s="14" t="inlineStr"/>
+      <c r="B52" s="24" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>Le rendu devenait poussif avec les 39 000 bougies par série : Scatter redessinait un marqueur par point à chaque zoom. Passage à SignalXY, qui ne trace que la partie visible, et recherche du point survolé limitée à une fenêtre trouvée par dichotomie au lieu de reprojeter toute la série. Les couleurs viennent maintenant d'une palette indexée sur la position de la série, pour que masquer une courbe ne recolore plus les autres. 🤖 Generated with Codebuff Co-Authored-By: Codebuff &lt;noreply@codebuff.com&gt;</t>
+        </is>
+      </c>
+      <c r="D52" s="14" t="inlineStr">
+        <is>
+          <t>[40]</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
+      <c r="A53" s="14" t="inlineStr"/>
+      <c r="B53" s="15" t="inlineStr"/>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>fusion branche 'main' of https://github.com/BlackAngelTVdev/P-Fun</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>[?]</t>
+        </is>
+      </c>
+      <c r="E53" s="14" t="inlineStr">
+        <is>
+          <t>[?]</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr"/>
+      <c r="B54" s="24" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>Le rendu devenait poussif avec les 39 000 bougies par série : Scatter redessinait un marqueur par point à chaque zoom. Passage à SignalXY, qui ne trace que la partie visible, et recherche du point survolé limitée à une fenêtre trouvée par dichotomie au lieu de reprojeter toute la série. Les couleurs viennent maintenant d'une palette indexée sur la position de la série, pour que masquer une courbe ne recolore plus les autres. 🤖 Generated with Codebuff Co-Authored-By: Codebuff &lt;noreply@codebuff.com&gt;</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>[?]</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
+          <t>[?]</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr"/>
+      <c r="B55" s="17" t="inlineStr"/>
+      <c r="C55" s="18" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="D55" s="18" t="inlineStr">
+        <is>
+          <t>1h31 (91 min)</t>
+        </is>
+      </c>
+      <c r="E55" s="17" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E53"/>
+  <autoFilter ref="A1:E56"/>
   <mergeCells count="7">
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A20:E20"/>
@@ -6101,7 +7550,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>13h57</t>
+          <t>14h38</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -6137,7 +7586,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2h20</t>
+          <t>2h26</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -6218,14 +7667,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>91</v>
       </c>
       <c r="C7" t="n">
-        <v>0.83</v>
+        <v>1.52</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0h50</t>
+          <t>1h31</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -6234,7 +7683,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>13.95</v>
+        <v>14.63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
doc(rapport): update du rapport
[35][WIP]
</commit_message>
<xml_diff>
--- a/doc/journal_de_travail.xlsx
+++ b/doc/journal_de_travail.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$7</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -56,7 +56,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -177,6 +177,18 @@
         <bgColor rgb="00558B2F"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C62828"/>
+        <bgColor rgb="00C62828"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004527A0"/>
+        <bgColor rgb="004527A0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -190,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -244,6 +256,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4221,7 +4239,6 @@
 
 <file path=xl/charts/chart39.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -4520,6 +4537,469 @@
 </file>
 
 <file path=xl/charts/chart40.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart41.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart42.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart43.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart44.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -6086,6 +6566,94 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="41" name="Chart 41"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId41"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="42" name="Chart 42"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId42"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="43" name="Chart 43"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId43"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="44" name="Chart 44"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId44"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -6378,7 +6946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="1"/>
@@ -7305,12 +7873,12 @@
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>[1]</t>
+          <t>[?]</t>
         </is>
       </c>
       <c r="E50" s="14" t="inlineStr">
         <is>
-          <t>[DONE]</t>
+          <t>[?]</t>
         </is>
       </c>
     </row>
@@ -7347,12 +7915,12 @@
       </c>
       <c r="D52" s="14" t="inlineStr">
         <is>
-          <t>[40]</t>
+          <t>[?]</t>
         </is>
       </c>
       <c r="E52" s="14" t="inlineStr">
         <is>
-          <t>[DONE]</t>
+          <t>[?]</t>
         </is>
       </c>
     </row>
@@ -7377,51 +7945,120 @@
     </row>
     <row r="54">
       <c r="A54" s="14" t="inlineStr"/>
-      <c r="B54" s="24" t="inlineStr">
-        <is>
-          <t>Performance</t>
+      <c r="B54" s="19" t="inlineStr">
+        <is>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C54" s="14" t="inlineStr">
         <is>
-          <t>Le rendu devenait poussif avec les 39 000 bougies par série : Scatter redessinait un marqueur par point à chaque zoom. Passage à SignalXY, qui ne trace que la partie visible, et recherche du point survolé limitée à une fenêtre trouvée par dichotomie au lieu de reprojeter toute la série. Les couleurs viennent maintenant d'une palette indexée sur la position de la série, pour que masquer une courbe ne recolore plus les autres. 🤖 Generated with Codebuff Co-Authored-By: Codebuff &lt;noreply@codebuff.com&gt;</t>
+          <t>mise a jour du rapport et du JNR</t>
         </is>
       </c>
       <c r="D54" s="14" t="inlineStr">
         <is>
-          <t>[?]</t>
+          <t>[10]</t>
         </is>
       </c>
       <c r="E54" s="14" t="inlineStr">
         <is>
-          <t>[?]</t>
+          <t>[DONE]</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="17" t="inlineStr"/>
-      <c r="B55" s="17" t="inlineStr"/>
-      <c r="C55" s="18" t="inlineStr">
-        <is>
-          <t>Total du jour</t>
-        </is>
-      </c>
-      <c r="D55" s="18" t="inlineStr">
-        <is>
-          <t>1h31 (91 min)</t>
-        </is>
-      </c>
-      <c r="E55" s="17" t="inlineStr"/>
+      <c r="A55" s="14" t="inlineStr"/>
+      <c r="B55" s="21" t="inlineStr">
+        <is>
+          <t>Refactorisation</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>verification linq</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>[30]</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
+      <c r="A56" s="14" t="inlineStr"/>
+      <c r="B56" s="25" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>fait que ca écrase les encien si chevauchement</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>[25]</t>
+        </is>
+      </c>
+      <c r="E56" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="14" t="inlineStr"/>
+      <c r="B57" s="26" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>ajout 2 tests</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>[25]</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="inlineStr"/>
+      <c r="B58" s="17" t="inlineStr"/>
+      <c r="C58" s="18" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="inlineStr">
+        <is>
+          <t>2h20 (140 min)</t>
+        </is>
+      </c>
+      <c r="E58" s="17" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E56"/>
+  <autoFilter ref="A1:E59"/>
   <mergeCells count="7">
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A20:E20"/>
@@ -7550,7 +8187,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>14h38</t>
+          <t>15h27</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -7586,7 +8223,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2h26</t>
+          <t>2h34</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -7667,14 +8304,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>91</v>
+        <v>140</v>
       </c>
       <c r="C7" t="n">
-        <v>1.52</v>
+        <v>2.33</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1h31</t>
+          <t>2h20</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -7683,7 +8320,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>14.63</v>
+        <v>15.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
doc(Rapport): ajout des maquettes et finalisation
[20][DONE]
</commit_message>
<xml_diff>
--- a/doc/journal_de_travail.xlsx
+++ b/doc/journal_de_travail.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -479,6 +479,237 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charge par jour (heures)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$C$2:$C$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumul des heures</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Tableau de bord'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Tableau de bord'!$A$2:$A$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Tableau de bord'!$J$2:$J$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <smooth val="1"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Heures</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
@@ -590,7 +821,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -786,6 +1017,50 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1083,7 +1358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2363,29 +2638,75 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="6" t="inlineStr"/>
-      <c r="B68" s="6" t="inlineStr"/>
-      <c r="C68" s="7" t="inlineStr">
+      <c r="A68" s="3" t="inlineStr"/>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Tâche</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>maj</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>[1]</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr"/>
+      <c r="B69" s="9" t="inlineStr">
+        <is>
+          <t>Fonctionnalité</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>double échelle</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>[40]</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>[WIP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr"/>
+      <c r="B70" s="6" t="inlineStr"/>
+      <c r="C70" s="7" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D68" s="7" t="inlineStr">
-        <is>
-          <t>2h02 (122 min)</t>
-        </is>
-      </c>
-      <c r="E68" s="6" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr"/>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>2h43 (163 min)</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E69"/>
+  <autoFilter ref="A1:E71"/>
   <mergeCells count="7">
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A62:E62"/>
@@ -2514,7 +2835,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>18h06</t>
+          <t>18h47</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -2550,7 +2871,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2h35</t>
+          <t>2h41</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -2657,14 +2978,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>122</v>
+        <v>163</v>
       </c>
       <c r="C8" t="n">
-        <v>2.03</v>
+        <v>2.72</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2h02</t>
+          <t>2h43</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -2673,7 +2994,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>18.1</v>
+        <v>18.78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Chore(release): Generation des pdf
[1][DONE]
</commit_message>
<xml_diff>
--- a/doc/journal_de_travail.xlsx
+++ b/doc/journal_de_travail.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Tableau de bord" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$E$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tableau de bord'!$A$1:$D$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42,7 +42,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -121,6 +121,12 @@
         <bgColor rgb="00558B2F"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F57F17"/>
+        <bgColor rgb="00F57F17"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -134,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -167,6 +173,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -283,12 +292,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
+              <f>'Tableau de bord'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$C$2:$C$8</f>
+              <f>'Tableau de bord'!$C$2:$C$10</f>
             </numRef>
           </val>
         </ser>
@@ -402,12 +411,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
+              <f>'Tableau de bord'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$J$2:$J$8</f>
+              <f>'Tableau de bord'!$J$2:$J$10</f>
             </numRef>
           </val>
         </ser>
@@ -479,6 +488,7 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -514,12 +524,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
+              <f>'Tableau de bord'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$C$2:$C$8</f>
+              <f>'Tableau de bord'!$C$2:$C$10</f>
             </numRef>
           </val>
         </ser>
@@ -623,246 +633,14 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
           <cat>
             <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
+              <f>'Tableau de bord'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Tableau de bord'!$J$2:$J$8</f>
-            </numRef>
-          </val>
-        </ser>
-        <smooth val="1"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Date</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Heures</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Charge par jour (heures)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Tableau de bord'!C1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Tableau de bord'!$C$2:$C$8</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Date</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Heures</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Cumul des heures</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Tableau de bord'!J1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Tableau de bord'!$A$2:$A$8</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Tableau de bord'!$J$2:$J$8</f>
+              <f>'Tableau de bord'!$J$2:$J$10</f>
             </numRef>
           </val>
         </ser>
@@ -1017,50 +795,6 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId4"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>12</col>
-      <colOff>0</colOff>
-      <row>7</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5760000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="5" name="Chart 5"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId5"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>12</col>
-      <colOff>0</colOff>
-      <row>25</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5760000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="6" name="Chart 6"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1358,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2433,7 +2167,7 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Le rendu devenait poussif avec les 39 000 bougies par série : Scatter redessinait un marqueur par point à chaque zoom. Passage à SignalXY, qui ne trace que la partie visible, et recherche du point survolé limitée à une fenêtre trouvée par dichotomie au lieu de reprojeter toute la série. Les couleurs viennent maintenant d'une palette indexée sur la position de la série, pour que masquer une courbe ne recolore plus les autres. 🤖 Generated with Codebuff Co-Authored-By: Codebuff &lt;noreply@codebuff.com&gt;</t>
+          <t>Le rendu devenait poussif avec les 39 000 bougies par série : Scatter redessinait un marqueur par point à chaque zoom. Passage à SignalXY, qui ne trace que la partie visible, et recherche du point survolé limitée à une fenêtre trouvée par dichotomie au lieu de reprojeter toute la série. Les couleurs viennent maintenant d'une palette indexée sur la position de la série, pour que masquer une courbe ne recolore plus les autres.</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -2684,37 +2418,278 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="6" t="inlineStr"/>
-      <c r="B70" s="6" t="inlineStr"/>
-      <c r="C70" s="7" t="inlineStr">
+      <c r="A70" s="3" t="inlineStr"/>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Tâche</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>mise a jour</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr"/>
+      <c r="B71" s="6" t="inlineStr"/>
+      <c r="C71" s="7" t="inlineStr">
         <is>
           <t>Total du jour</t>
         </is>
       </c>
-      <c r="D70" s="7" t="inlineStr">
-        <is>
-          <t>2h43 (163 min)</t>
-        </is>
-      </c>
-      <c r="E70" s="6" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr"/>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>2h45 (165 min)</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr"/>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Tâche</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Ajouter un commentaire d'évaluation à 80%</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>[?]</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr"/>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Tâche</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Ajout de questions pour validation de maîtrise</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>[?]</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr"/>
+      <c r="B76" s="4" t="inlineStr"/>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Ratrapage de teste</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>[180]</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr"/>
+      <c r="B77" s="6" t="inlineStr"/>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>3h00 (180 min)</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr"/>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>ajout des maquettes et finalisation</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>[20]</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr"/>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>[5]</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr"/>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Tâche</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>ajoutes des data d'example</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>[DONE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr"/>
+      <c r="B83" s="14" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>je ne comprend pas encoer le code mais je push psk pas le choix</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>[?]</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>[?]</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr"/>
+      <c r="B84" s="6" t="inlineStr"/>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>0h27 (27 min)</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E71"/>
-  <mergeCells count="7">
+  <autoFilter ref="A1:E85"/>
+  <mergeCells count="10">
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A62:E62"/>
     <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A73:E73"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A78:E78"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A47:E47"/>
     <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A79:E79"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2726,7 +2701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2766,12 +2741,12 @@
           <t>Valeur</t>
         </is>
       </c>
-      <c r="I1" s="14" t="inlineStr">
+      <c r="I1" s="15" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="J1" s="14" t="inlineStr">
+      <c r="J1" s="15" t="inlineStr">
         <is>
           <t>Cumul (h)</t>
         </is>
@@ -2794,13 +2769,13 @@
           <t>2h57</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
+      <c r="F2" s="15" t="inlineStr">
         <is>
           <t>Jours suivis</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -2828,14 +2803,14 @@
           <t>3h00</t>
         </is>
       </c>
-      <c r="F3" s="14" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>Temps total</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>18h47</t>
+          <t>22h16</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -2864,14 +2839,14 @@
           <t>1h15</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>Moyenne / jour</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2h41</t>
+          <t>2h28</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -2900,7 +2875,7 @@
           <t>2h56</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>Jour le plus chargé</t>
         </is>
@@ -2978,14 +2953,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C8" t="n">
-        <v>2.72</v>
+        <v>2.75</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2h43</t>
+          <t>2h45</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -2994,11 +2969,63 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>18.78</v>
+        <v>18.82</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>180</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>3h00</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>21.82</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>27</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0h27</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>22.27</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D8"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>